<commit_message>
added cache locking for improved performance
</commit_message>
<xml_diff>
--- a/wf1.xlsx
+++ b/wf1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,33 +516,34 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Laura Silvester
-Name: Laura Silvester
-Location: Vancouver, British Columbia, Canada
-Company: Anthill
-Company Location: Chicago, IL, United States
-Title: Co-founder, Chief Operating Officer &amp; Head of Product
-Industry: Computer Software
-Education: Bachelor of Commerce with a minor in English Literature from UBC Sauder School of Business; additional training from Product Institute (Product Management), Female Funders Angel Academy (Investor Accelerator Program), and Bader College (Honours, Bachelor of Arts).
-Email: No personal email found; company contact email is partnerships@anthill.co
-Phone: No personal phone number found
-Website: http://www.anthill.co
-LinkedIn: https://ca.linkedin.com/in/laurasilvester
-Company LinkedIn: https://www.linkedin.com/company/29309264
-Summary: Laura is a technology executive and entrepreneur focused on AI-powered workforce management solutions for frontline workers. She co-founded Anthill, which automates workflows to recruit, onboard, manage, and retain frontline workforces in 75 languages. She has held senior leadership roles at Hootsuite and lululemon and is recognized for leadership in technology and business. She is active in advisory and volunteer roles related to education, AI, and startups. Anthill is headquartered in Chicago, IL, with offices in Vancouver and other locations. The company specializes in AI solutions for high-volume, hard-to-reach frontline workforces, emphasizing responsible AI use and workforce empowerment.
-Social Media: TikTok profile exists but with minimal activity; Instagram profile snapshot not ready.
-Awards: Recognized in Business in Vancouver's Forty Under 40 Awards and The Peak's 2023 Emerging Leaders List.
-References to verify identity include company affiliation, location, education, and leadership roles, confirming this is the correct Laura Silvester.</t>
+          <t>Person: Laura Silvester
+- Name: Laura Silvester
+- Age: 37
+- Location: Vancouver, BC, Canada (based on article and local references)
+- Company: Anthill AI
+- Title: Co-founder and Chief Operating Officer (COO)
+- Industry: Technology, specifically workforce management software for frontline workers
+- Education: Commerce degree with a minor in English Literature (specific university not explicitly stated in this article, but previous notes indicate UBC Sauder School of Business alumni involvement)
+- Notable achievements: Recognized in Business in Vancouver's Forty Under 40 Awards, highlighting her leadership and impact in technology and business.
+- Personal insights: Values trust in business, leadership as showing up authentically, and balances family life with career. Has a passion for Shakespeare and local community spots in Vancouver.
+- Company website: https://www.anthill.co
+- Location details: Although the initial input mentioned Chicago, IL, the article and other sources place her in Vancouver, BC, Canada, which aligns with Anthill AI's base and her local community involvement.
+- No direct email or phone number found in this source.
+This profile matches the LinkedIn URL provided and the company Anthill AI, confirming the correct individual. The article provides rich qualitative data about her leadership style, values, and recognition in the tech industry.
+References:
+- Business in Vancouver article: https://www.biv.com/news/technology/biv-forty-under-40-awards-laura-silvester-11632004
+- Anthill AI website: https://www.anthill.co
+- LinkedIn profile: https://ca.linkedin.com/in/laurasilvester</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{"http://www.anthill.co": "Anthill company website detailing the AI-powered frontline workforce management platform, company location in Chicago, IL, and contact information.", "https://ca.linkedin.com/in/laurasilvester": "Laura Silvester's LinkedIn profile showing her current role as Co-founder, COO, and Head of Product at Anthill, education background, and professional experience.", "https://ventureforcanada.ca/about-us/our-people/laura-silvester": "Profile of Laura Silvester on Venture For Canada website confirming her role at Anthill and leadership experience.", "https://www.biv.com/news/technology/biv-forty-under-40-awards-laura-silvester-11632004": "Business in Vancouver article recognizing Laura Silvester in the Forty Under 40 Awards.", "https://www.linkedin.com/company/29309264": "Anthill's LinkedIn company profile confirming company details, industry, and headquarters location."}</t>
+          <t>{"http://www.anthill.co": "Official website of Anthill, the company co-founded by Laura Silvester, providing context on company industry and headquarters location.", "https://alumni.ubc.ca/about/board": "UBC Alumni Association board page listing Laura Silvester as a board member and alumni leader.", "https://ca.linkedin.com/in/laurasilvester": "LinkedIn profile of Laura Silvester, confirming her professional role and affiliations.", "https://www.anthill.co": "Official website of Anthill AI, the company co-founded by Laura Silvester, specializing in workforce management technology.", "https://www.anthill.co/about": "Anthill company website providing details about the company, leadership, and contact information.", "https://www.biv.com/news/technology/biv-forty-under-40-awards-laura-silvester-11632004": "Business in Vancouver article profiling Laura Silvester as a Forty Under 40 award winner, detailing her role as Co-founder and COO of Anthill AI, her leadership philosophy, education, and personal background."}</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>{"company": "Anthill (Anthill AI)", "content": "Original lead information: { company: Chicago, IL, United States; linkedin: https://ca.linkedin.com/in/laurasilvester; location: Anthill; name: Laura Silvester }\n\nSummary of findings: Laura Silvester is co-founder, COO and Head of Product at Anthill (Anthill AI). She is based in Vancouver, British Columbia (personal location) while Anthill is headquartered in Chicago, IL. Education includes UBC Sauder School of Business (Bachelor of Commerce, minor in English Literature), Product Institute (Product Management), Female Funders Angel Academy, and Bader College. No personal email or phone number publicly available. Company contact: partnerships@anthill.co. Key references: https://ca.linkedin.com/in/laurasilvester ; http://www.anthill.co ; https://www.linkedin.com/company/29309264 ; https://www.biv.com/news/technology/biv-forty-under-40-awards-laura-silvester-11632004 ; https://ventureforcanada.ca/about-us/our-people/laura-silvester.", "education": "Bachelor of Commerce (Commerce) with a minor in English Literature — UBC Sauder School of Business; Product Institute (Product Management); Female Funders Angel Academy (Angel Academy / Investor Accelerator); Bader College (Honours, Bachelor of Arts)", "email": "", "industry": "Computer Software (AI-powered frontline workforce management)", "linkedin": "https://ca.linkedin.com/in/laurasilvester", "location": "Vancouver, British Columbia, Canada (individual); Chicago, IL, United States (Anthill HQ)", "name": "Laura Silvester", "phone": "", "title": "Co-founder, Chief Operating Officer &amp; Head of Product", "website": "http://www.anthill.co"}</t>
+          <t>{"company": "Anthill", "content": "Original lead information: {company: Chicago, IL, United States; linkedin: https://ca.linkedin.com/in/laurasilvester; location: Anthill; name: Laura Silvester}\nSummary: Laura Silvester is co-founder, COO and Head of Product at Anthill, an AI-driven frontline workforce automation company headquartered in Chicago with operations in Vancouver. No personal email or phone number was publicly available. Education and prior roles (UBC Sauder BCom, Hootsuite, Lululemon, McKinsey) are confirmed across LinkedIn, Anthill site and news sources.\nKey references:\n- LinkedIn: https://ca.linkedin.com/in/laurasilvester\n- Anthill (company): https://www.anthill.co/ and https://www.anthill.co/about\n- Business in Vancouver profile: https://www.biv.com/news/technology/biv-forty-under-40-awards-laura-silvester-11632004\n- UBC Alumni board listing: https://alumni.ubc.ca/about/board\nNote: company partnership contact found publicly (partnerships@anthill.co) but no personal contact for Laura. No further next steps required to validate identity; additional research could target corporate press releases or UBC alumni directories if a direct email is required.", "education": "Bachelor of Commerce (BCom), UBC Sauder School of Business (graduated 2011) — Finance &amp; English Literature; Product Institute (Product Management); Female Funders Angel Academy; Bader College (Honours)", "email": "", "industry": "Computer software / Workforce management technology (AI-driven frontline workforce automation, HR software)", "linkedin": "https://ca.linkedin.com/in/laurasilvester", "location": "Vancouver, British Columbia, Canada (personal); Anthill HQ: Chicago, IL, United States", "name": "Laura Silvester", "phone": "", "title": "Co-founder; Chief Operating Officer (COO) &amp; Head of Product", "website": "https://www.anthill.co"}</t>
         </is>
       </c>
     </row>
@@ -572,11 +573,488 @@
           <t>https://www.linkedin.com/in/yj87</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Person: Young-Jae Kim
+- Full Name: Young-Jae Kim
+- Location: Greater Chicago Area, Chicago, IL, United States
+- Current Company: Anthill AI
+- Company Website: https://www.anthill.co
+- Company Address: 111 W Illinois Street, Suite 500, Chicago, IL 60654
+- Job Title: Co-founder &amp; Chief Strategy Officer (CSO)
+- Industry: Human Resources and Computer Software
+- Education:
+  - PhD in Industrial-Organizational Psychology, The University of Georgia (2015-2020)
+  - MS in Organizational Behavior and Management Science, Korea Advanced Institute of Science and Technology (KAIST) (2013-2014)
+  - BS in Psychology, University of Illinois Urbana-Champaign
+- Previous Experience:
+  - Senior Analyst at Assesta, Co. Ltd., Seoul, Korea
+  - IO Psychology Consultant at Pinsight, Denver, CO
+  - HR Analyst at LG CNS Co., Ltd., Seoul, Korea
+- LinkedIn Profile: https://www.linkedin.com/in/yj87
+- Company Description: Anthill AI provides AI-powered frontline workforce management solutions, automating recruitment, onboarding, management, and retention of frontline workers in 75 languages. The company is SOC 2 Type II, HIPAA, and GDPR compliant.
+- Company Industry: Computer Software
+- Company Size: Approximately 11 employees
+- Company Revenue: Approx. $595,000
+- Company Headquarters: Chicago, IL, USA
+- Contact Email (Company): partnerships@anthill.co
+- Recognitions: Featured in Forbes, TechCrunch, and other notable publications
+- Social Media: Active on LinkedIn with 500+ connections and 927 followers
+- Skills: Data Analysis, Statistics, Research Design, Survey Design, Experimental Design, Text Mining, R, SAS, Mplus, HLM, SPSS, KNIME, SQL, NetLogo
+- Summary: Young-Jae Kim is an AI expert and people scientist focused on transforming workforce management for frontline teams through AI technology at Anthill AI. He has extensive experience in industrial-organizational psychology and human resources.
+No personal email or phone number publicly available.
+References:
+- LinkedIn profile: https://www.linkedin.com/in/yj87
+- Anthill AI website: https://www.anthill.co
+- University of Georgia: https://www.linkedin.com/company/166638/
+- Pinsight: http://www.pinsight.com
+- LG CNS: https://www.lgcns.com/kr
+This profile matches the source of truth data with location Chicago, IL, LinkedIn URL, and company Anthill AI, confirming the correct individual.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>{"http://www.anthill.co": "Official website of Anthill AI, the company where Young-Jae Kim is Co-founder &amp; CSO, specializing in AI-powered workforce management solutions.", "http://www.pinsight.com": "Website of Pinsight, previous employer of Young-Jae Kim as IO Psychology Consultant.", "https://www.anthill.co": "Official website of Anthill AI, company co-founded by Young-Jae Kim, providing AI-powered frontline workforce management solutions.", "https://www.bloomberg.com/profile/company/1839938D:US": "Bloomberg company profile for Anthill AI Inc, providing company overview, industry, and contact information.", "https://www.crunchbase.com/person/young-jae-kim": "Crunchbase profile confirming education background and role at Anthill AI.", "https://www.lgcns.com/kr": "Website of LG CNS, previous employer of Young-Jae Kim as HR Analyst.", "https://www.linkedin.com/company/166638": "LinkedIn page for The University of Georgia, where Young-Jae Kim earned his PhD.", "https://www.linkedin.com/in/yj87": "LinkedIn profile of Young-Jae Kim, confirming current role, education, and location."}</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>{"company": "Anthill AI (Anthill AI, Inc.)", "content": "Original lead information:\ncontent:\n  company: Chicago, IL, United States\n  linkedin: https://www.linkedin.com/in/yj87\n  location: Anthill\n  name: Young-Jae Kim\n\nSummary of research &amp; references:\n- Confirmed LinkedIn profile: https://www.linkedin.com/in/yj87 (Co-founder &amp; CSO at Anthill AI; education and prior roles listed)\n- Company website: https://www.anthill.co (Anthill AI — company HQ in Chicago, IL; company contact: partnerships@anthill.co)\n- Crunchbase &amp; Bloomberg listings corroborate role, company details and education\n\nNotes:\n- No personal email or phone number was found in public sources. Company contact email (general) is partnerships@anthill.co but this is a company-level contact, not an individual address.\n- Title has minor variations in sources (Co-founder &amp; CSO / Chief Strategy Officer; one source briefly referenced CTO) — primary, consistent title used above.\n\nKey references:\n- LinkedIn profile: https://www.linkedin.com/in/yj87\n- Anthill AI (official site): https://www.anthill.co\n- Crunchbase person profile: https://www.crunchbase.com/person/young-jae-kim\n- Bloomberg company profile: https://www.bloomberg.com/profile/company/1839938D:US", "education": "PhD in Industrial-Organizational Psychology, The University of Georgia; MS in Organizational Behavior and Management Science, Korea Advanced Institute of Science and Technology (KAIST); BS in Psychology, University of Illinois Urbana-Champaign", "email": "", "industry": "Human Resources; Computer Software (AI-powered frontline workforce management)", "linkedin": "https://www.linkedin.com/in/yj87", "location": "Greater Chicago Area (Chicago, IL, United States)", "name": "Young-Jae Kim", "phone": "", "title": "Co-founder &amp; Chief Strategy Officer (CSO)", "website": "https://www.anthill.co"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jishai Evers</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Archetype Labs</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>jishai@archetype.do</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>New York, NY, United States</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://il.linkedin.com/in/jishai</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Person: Jishai Evers
+Name: Jishai Evers
+Location: New York, NY, United States (company location), also associated with Tel Aviv, Israel
+Company: Archetype Labs (venture builder for AI products), also Co-Founder &amp; Chief Product Officer at Headroom AI
+Title: Co-Founder &amp; Chief Product Officer (CPO) at Archetype Labs and Headroom AI
+LinkedIn: https://il.linkedin.com/in/jishai
+Website: https://headroom.com (Headroom AI company website), personal site jishaievers.com
+Industry: AI software, SaaS for SMBs, tech startups, AI-powered productivity tools
+Education: Economics degree from University of Amsterdam; Law degree from Bar-Ilan University; additional Hebrew studies at Ulpan Akiva
+Email: Not publicly found
+Phone: Not publicly found
+Professional Summary: Serial entrepreneur and product leader with over a decade of experience in AI, data visualization, media, and enterprise software. Former Product Lead at Palantir Technologies. Founder of multiple startups including Headroom AI, Rubber Duck Bath Party (NFT project), Dadaviz, and WikiBrains. Known for hands-on product development and innovative AI integration. Active on X (Twitter) as @Jishai with professional updates and community engagement.
+References to patents exist but the patent link provided returned a 404 error.
+No public email or phone number was found in the resources.
+The LinkedIn profile and company website provide the most reliable and up-to-date information.
+The X profile (@Jishai) confirms his current roles and interests in AI, startups, and product building.
+Overall, the data confirms the lead is the correct Jishai Evers associated with Archetype Labs and Headroom AI in New York.
+Relevant URLs:
+- LinkedIn: https://il.linkedin.com/in/jishai
+- Company website: https://headroom.com
+- Twitter/X: https://x.com/Jishai
+- Personal website: jishaievers.com
+Findings:
+- Jishai Evers is a Co-Founder and CPO at Archetype Labs and Headroom AI.
+- Based in New York, with strong ties to Tel Aviv and Amsterdam.
+- Holds degrees in Economics and Law.
+- Experienced in AI, SaaS, product leadership, and startup founding.
+- Active on social media with a professional focus.
+- No public contact email or phone number found.
+- Company website and LinkedIn profile are primary sources for current info.
+Next Steps:
+- None needed as sufficient information has been gathered to fill the required fields.
+- Monitor LinkedIn and Twitter for any future updates or contact info disclosures.
+- If contact details become necessary, consider reaching out via LinkedIn messaging or company contact forms.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>{"https://headroom.com": "Company website for Headroom AI, co-founded by Jishai Evers, providing information about the company and its AI software products.", "https://headroom.com/?utm_source=linkedin&amp;utm_medium=social&amp;utm_campaign=bio": "Company website for Headroom (Archetype Labs), providing AI-powered software solutions for SMBs, confirming company details and industry.", "https://il.linkedin.com/in/jishai": "LinkedIn profile of Jishai Evers confirming current roles, education, and professional background.", "https://ppubs.uspto.gov/dirsearch-public/patents/html/20230153095?source=US-PGPUB": "Patent titled 'SEAMLESS SYNCHRONIZATION ACROSS DIFFERENT APPLICATIONS' issued to Jishai Evers.", "https://www.crunchbase.com/person/jishai-evers": "Crunchbase profile summarizing Jishai's career and company affiliations.", "https://www.linkedin.com/company/91102183": "LinkedIn company page for Archetype Labs, not publicly accessible without login.", "https://x.com/Jishai": "X (Twitter) profile of Jishai Evers showing professional activity, interests in AI, startups, and product building.", "jishaievers.com": "Personal website of Jishai Evers with professional bio and background information."}</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>{"company": "Archetype Labs (Headroom / Headroom AI)", "content": "Original lead information:\ncontent:\n  company: New York, NY, United States\n  linkedin: https://il.linkedin.com/in/jishai\n  location: Archetype Labs\n  name: Jishai Evers\n\nSummary of findings (most relevant facts):\n- Full name: Jishai Evers\n- Current company: Archetype Labs (operating product/brand: Headroom / Headroom AI)\n- Current title: Co‑Founder &amp; Chief Product Officer (CPO) at Archetype Labs (since May 2023)\n- Location: personal LinkedIn location in Israel (Tel Aviv area reported in sources); company HQ associated with New York, NY, United States\n- Industry: Computer software / AI (SaaS for SMBs)\n- Education: degrees from University of Amsterdam and Bar‑Ilan University; intensive Hebrew course at Ulpan Akiva\n- Previous notable roles: Product Lead at Palantir Technologies (2017–2022); VP Product at Vocativ; founder/cofounder of multiple startups (dadaviz, WikiBrains, etc.)\n- Public contact info: no verified public email or phone discovered\n\nPrimary references used:\n- LinkedIn profile: https://il.linkedin.com/in/jishai\n- Company / product website: https://headroom.com (Headroom / Archetype Labs)\n- X (Twitter) profile: https://x.com/Jishai\n- Patent/publication reference: https://ppubs.uspto.gov/dirsearch-public/patents/html/20230153095?source=US-PGPUB\n- Personal site (as referenced): jishaievers.com\n- Archetype Labs (LinkedIn company page reference): https://www.linkedin.com/company/91102183/\n- Crunchbase person page (referenced; may be inaccessible): https://www.crunchbase.com/person/jishai-evers\n\nNotes: Email and phone left blank because no reliable, complete public contact details were found. LinkedIn and the company website are the primary authoritative sources for role and company.", "education": "BSc / LL.B (Economics &amp; Law), University of Amsterdam (2010–2011); BSc (Economics, Political Science &amp; Sociology), Bar‑Ilan University (2009–2010); Intensive Hebrew course, Ulpan Akiva (2009)", "email": "", "industry": "Computer Software / AI (SaaS for SMBs)", "linkedin": "https://il.linkedin.com/in/jishai", "location": "Based in Israel (personal location on LinkedIn); company HQ / associated location: New York, NY, United States", "name": "Jishai Evers", "phone": "", "title": "Co‑Founder &amp; Chief Product Officer (CPO) at Archetype Labs (Headroom) — since May 2023", "website": "https://headroom.com"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fifi Kara</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Aster Solutions, Inc.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>fifi@astercare.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, United States</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/fifikara</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Person: Fifi Kara
+- Full Name: Fifi Kara
+- Location: San Francisco Bay Area, California, United States
+- Current Company: Aster Solutions, Inc. (also known as Aster)
+- Company Website: https://astercare.com
+- Job Title: Co-Founder &amp; CEO (since June 2023)
+- Email: fifi@astercare.com (matches company domain astercare.com)
+- Industry: Hospital &amp; Health Care, focused on women's health technology
+- Company Description: Aster provides an AI-powered operating system for women's health clinics, active in over 15 U.S. states, supporting over 10,000 patients. The platform automates patient management from scheduling to charting to improve clinical efficiency and patient outcomes.
+- Company Size: Approximately 35 employees on LinkedIn
+- Company Funding: Raised $2.4 million in pre-seed funding
+- Education: Bachelor of Science (BSc) in Social Policy &amp; Government from The London School of Economics and Political Science (LSE); Fulbright Scholar at Indiana University Bloomington (Kelly School of Business); participated in Y Combinator Summer 2019 batch
+- Previous Experience: Product Design Manager at Meta (Facebook) in Health &amp; Fitness division; worked on AR/VR health products and consumer products like Messenger and Workrooms
+- Social Media Profiles:
+  - LinkedIn: https://www.linkedin.com/in/fifikara
+  - Instagram: https://www.instagram.com/fifikara
+  - TikTok: https://www.tiktok.com/@fifikara
+  - Twitter: https://twitter.com/FifiKara
+- Additional Notes: 
+  - Originally from London
+  - Over 10 years of experience developing consumer and B2B products across UK, Europe, and US
+  - Recognized for leadership and innovation in health technology
+  - No public phone number found
+This information is consistent across multiple sources and confirms the identity of Fifi Kara associated with Aster Solutions, Inc.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>{"https://astercare.com": "Company website for Aster Solutions, Inc., providing company overview and contact information.", "https://astercare.com/team/fifi": "Company team page with detailed bio of Fifi Kara, CEO of Aster.", "https://peopleofcolorintech.com/articles/aster-raises-2-4m-for-maternal-healthcare-platform-in-pre-seed-round-led-by-black-vcs": "News article confirming Aster's $2.4 million pre-seed funding round and company focus on maternal health.", "https://twitter.com/FifiKara": "Twitter profile of Fifi Kara, consistent with professional identity.", "https://www.astercare.com/team/fifi": "Official Aster Solutions team page with detailed bio of Fifi Kara, CEO and Co-Founder.", "https://www.instagram.com/fifikara": "Instagram profile of Fifi Kara.", "https://www.linkedin.com/company/3325": "LinkedIn page for Indiana University Bloomington, where Fifi Kara was a Fulbright Scholar.", "https://www.linkedin.com/company/6544": "LinkedIn page for The London School of Economics and Political Science (LSE), where Fifi Kara earned her BSc degree.", "https://www.linkedin.com/in/fifikara": "LinkedIn profile of Fifi Kara confirming current role, education, and previous experience.", "https://www.tiktok.com/@fifikara": "TikTok profile of Fifi Kara.", "https://www.ycombinator.com/verify/zqlcy9z0f4rtbfsn": "Y Combinator verification of Fifi Kara's participation in Summer 2019 batch."}</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>{"company": "Aster Solutions, Inc. (Aster)", "content": "Original lead information (unchanged):\ncontent:\n  company: San Francisco, CA, United States\n  linkedin: https://www.linkedin.com/in/fifikara\n  location: Aster Solutions, Inc.\n  name: Fifi Kara\n  title: fifi@astercare.com\n\nSummary of findings (sources: LinkedIn, Aster team page, Y Combinator verification, news coverage, social media):\n- Fifi Kara is Co-Founder &amp; CEO of Aster Solutions, Inc. (Aster), headquartered in the San Francisco Bay Area. Company site: https://astercare.com\n- Email observed on company domain: fifi@astercare.com (matches company domain astercare.com and company team page).\n- Education: BSc Social Policy &amp; Government (LSE); Fulbright Scholar at Indiana University Bloomington; Y Combinator S19 alum.\n- Industry: Health tech focused on women's and maternal health (Hospital &amp; Health Care, Femtech).\n- No public phone number located in available sources.\n\nKey reference URLs:\n- LinkedIn profile: https://www.linkedin.com/in/fifikara\n- Aster company site: https://astercare.com\n- Aster team bio (Fifi): https://astercare.com/team/fifi\n- Y Combinator verification: https://www.ycombinator.com/verify/zqlcy9z0f4rtbfsn\n- News coverage (funding &amp; company focus): https://peopleofcolorintech.com/articles/aster-raises-2-4m-for-maternal-healthcare-platform-in-pre-seed-round-led-by-black-vcs/\n- Twitter: https://twitter.com/FifiKara\n- Instagram: https://www.instagram.com/fifikara\n- TikTok: https://www.tiktok.com/@fifikara\n\nNext steps to locate missing phone or verify additional contact info (exact URLs/tools recommended):\n1) Check Aster's website contact page or press kit for an office phone or PR contact: https://astercare.com (site contact/footer/team pages).\n2) Use business contact discovery services (Hunter.io, RocketReach, Lusha, Clearbit) to search fifi@astercare.com domain for phone entries (example: https://hunter.io/search/domain/astercare.com).\n3) Search company registration / California Secretary of State filings for Aster Solutions, Inc. for registered agent or phone: https://www.sos.ca.gov/business-programs/business-entities\n4) Review press releases and investor pages (venture firms named in coverage) for an ops/PR contact phone.\n5) If required, verify email via email-sending probe or email verification tool (Never send marketing without permission).\n\nIf you want further research (phone or deeper verification), I can run the above steps and attempt direct scraping of the Aster team page and relevant press releases.", "education": "BSc, Social Policy &amp; Government — London School of Economics and Political Science (LSE); Fulbright Scholar — Indiana University Bloomington (Entrepreneurship); Y Combinator, Summer 2019 (S19) alum", "email": "fifi@astercare.com", "industry": "Hospital &amp; Health Care; Health Tech; Femtech; Women's &amp; Maternal Health", "linkedin": "https://www.linkedin.com/in/fifikara", "location": "San Francisco Bay Area, California, United States", "name": "Fifi Kara", "phone": "", "title": "Co-Founder &amp; CEO", "website": "https://astercare.com"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Dr. Lailah Kara-Newton</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Aster Solutions, Inc.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>lailah@astercare.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, United States</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/lailahkaranewton</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Person: Dr. Lailah Kara-Newton
+- Name: Dr. Lailah Kara-Newton
+- Location: San Francisco, CA, United States
+- Company: Aster Solutions, Inc.
+- LinkedIn: https://www.linkedin.com/in/lailahkaranewton
+- Title: Co-Founder &amp; Chief Medical Officer
+- Industry: Women's Health Technology / Health Tech
+- Education: Not explicitly stated in current resources; known as a practicing OB-GYN, implying medical degree and specialization in obstetrics and gynecology.
+- Email: Not publicly available from current resources.
+- Phone: Not publicly available from current resources.
+- Website: https://www.astercare.com (Company website for Aster Solutions, Inc.)
+Additional Context:
+- Dr. Lailah Kara-Newton is a practicing OB-GYN turned health tech founder.
+- She co-founded Aster, an AI-powered electronic health record (EHR) system specifically designed for women's healthcare.
+- Aster has supported over 250 births and is used in 70+ clinics.
+- The company focuses on improving provider efficiency and redefining pregnancy, postpartum, and women's wellness care delivery.
+- The podcast episode "Episode 40: You're Ignoring a $1 Trillion Opportunity" on TeqTalk features her discussing her mission and innovations.
+References:
+- Podcast episode on Apple Podcasts: https://podcasts.apple.com/us/podcast/episode-40-youre-ignoring-a-%241-trillion-opportunity/id1741536787?i=1000718828473
+- Company website: https://www.astercare.com
+- LinkedIn profile: https://www.linkedin.com/in/lailahkaranewton
+No direct contact information (email or phone) was found in the current resources.
+Findings are consistent with the source of truth input and confirm her role and company association.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>{"https://astercare.com": "Official website of Aster, the company co-founded by Dr. Lailah Kara-Newton, focused on AI-powered women's health solutions.", "https://femtechinsider.com/aster-seed-round": "News article reporting Aster Solutions, Inc.'s $2.4 million seed funding round and company mission in maternal health.", "https://podcasts.apple.com/us/podcast/episode-40-youre-ignoring-a-%241-trillion-opportunity/id1741536787?i=1000718828473": "Podcast episode featuring Dr. Lailah Kara-Newton discussing her work with Aster Solutions, Inc. and innovations in women's health technology.", "https://rocketreach.co/lailah-kara-newton-email_742992966": "RocketReach profile for Lailah Kara-Newton confirming role as Co-Founder and Chief Medical Officer at AsterCare, education background, and general contact info.", "https://www.astercare.com": "Official website of Aster Solutions, Inc., the company co-founded by Dr. Lailah Kara-Newton.", "https://www.linkedin.com/in/lailahkaranewton": "LinkedIn profile of Dr. Lailah Kara-Newton, confirming her role as Co-Founder &amp; Chief Medical Officer at Aster Solutions, Inc."}</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>{"company": "Aster Solutions, Inc. (Aster)", "content": "Original lead information: { company: San Francisco, CA, United States; linkedin: https://www.linkedin.com/in/lailahkaranewton; location: Aster Solutions, Inc.; name: Dr. Lailah Kara-Newton }\n\nSummary of findings: Dr. Lailah Kara-Newton is the Co-Founder &amp; Chief Medical Officer at Aster Solutions, Inc. (branded Aster), a San Francisco-based healthcare technology company focused on AI-enabled maternal and women’s health (EHR and voice AI agents). Educational background: MBBS from Barts and The London School of Medicine and Dentistry; BS in Global Public Health from Queen Mary University of London. No personal/individual email or phone number was found in public sources; company contact details are available on the corporate site. Key sources: LinkedIn profile and company website, plus coverage of Aster’s seed funding.\n\nUseful references:\n- LinkedIn (professional profile): https://www.linkedin.com/in/lailahkaranewton\n- Aster official website: https://www.astercare.com\n- News on seed funding and company mission: https://femtechinsider.com/aster-seed-round\n- RocketReach company/person listing (profile page): https://rocketreach.co/lailah-kara-newton-email_742992966\n- Podcast featuring Dr. Kara-Newton: https://podcasts.apple.com/us/podcast/episode-40-youre-ignoring-a-%241-trillion-opportunity/id1741536787?i=1000718828473\n\nNotes: Individual contact fields (email, phone) left empty because no reliable personal contact details were found in public sources. Company contact info (general) exists on the company website (hello@astercare.com; +1 415 874 1544).", "education": "MBBS, Barts and The London School of Medicine and Dentistry; BS in Global Public Health, Queen Mary University of London", "email": "", "industry": "Hospital &amp; Health Care; Healthcare Technology; Women's Health", "linkedin": "https://www.linkedin.com/in/lailahkaranewton", "location": "San Francisco, California, United States", "name": "Dr. Lailah Kara-Newton", "phone": "", "title": "Co-Founder &amp; Chief Medical Officer", "website": "https://astercare.com"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Daniel Faddoul</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Auditive, Inc.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>daniel.faddoul@auditive.io</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Walnut Creek, California, United States</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/danielfaddoul</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Daniel Faddoul
+Name: Daniel Faddoul
+Location: Walnut Creek, California, United States (San Francisco Bay Area)
+Company: Auditive, Inc.
+Company Website: https://www.auditive.io/
+Company Address: 1212 Broadway Plaza Suite 2100, Walnut Creek, CA 94596
+Title: Founder, CEO
+Industry: Internet / Computer Software (Third-party risk management software)
+LinkedIn: https://www.linkedin.com/in/danielfaddoul
+Email: daniel@auditive.io (confirmed business email)
+Phone: No confirmed personal phone number publicly available
+Education: 
+- Master of Finance (MFin), Princeton University (2009-2011)
+- Bachelor of Engineering (BEng) in Aeronautical Engineering, Imperial College London (2001-2005)
+- Lycee Francais Charles de Gaulle - London (1994-2001)
+Previous Employers: Goldman Sachs (Fixed Income Portfolio Management), Meta (Facebook) (Manager - New Products Analyst), Bain &amp; Company (Consultant), Doma (Senior Director of Product Management), One Concern (Product Manager)
+Company Funding: Auditive completed a seed funding round in July 2024 with investors including Everywhere Ventures and Wedbush Ventures
+Languages: English (native/bilingual), French (native/bilingual), Arabic (limited working proficiency), Spanish (limited working proficiency)
+Summary: Daniel is an experienced professional with over 16 years in finance, technology, and product management. He founded Auditive to transform third-party risk management using AI-powered continuous monitoring and onboarding solutions. Auditive's platform is designed to provide real-time clarity for security leaders and CISOs, replacing manual and inefficient processes.
+References include his LinkedIn profile, company website, Crunchbase funding data, and various professional profiles.
+This information aligns with the source of truth and confirms the correct identity and professional details of Daniel Faddoul.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>{"https://informaconnect.com/finovatespring/speakers/daniel-faddoul": "FinovateSpring speaker profile for Daniel Faddoul, confirming his position as Founder and CEO of Auditive and summarizing his professional background.", "https://meetings.hubspot.com/daniel-faddoul/auditive-demo": "Scheduling page for demos with Daniel Faddoul, confirming his role and contact point for Auditive.", "https://rocketreach.co/daniel-faddoul-email_758874530": "RocketReach profile providing Daniel Faddoul's contact information including emails and partial phone number, confirming his role as Founder and CEO at Auditive.", "https://www.auditive.io": "Official website of Auditive, the company founded by Daniel Faddoul, providing details about the company's products and contact information.", "https://www.crunchbase.com/organization/auditive": "Crunchbase profile for Auditive, showing company funding rounds and investors.", "https://www.linkedin.com/in/danielfaddoul": "LinkedIn profile of Daniel Faddoul, confirming his role as Founder and CEO of Auditive, education, and professional background."}</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>{"company": "Auditive, Inc.", "content": "Original lead information:\n- name: Daniel Faddoul\n- linkedin: https://www.linkedin.com/in/danielfaddoul\n- location: Auditive, Inc. / Walnut Creek, California, United States\n\nSummary of findings:\nDaniel Faddoul is the Founder &amp; CEO of Auditive, Inc., a Walnut Creek, CA–based SaaS company providing AI‑powered continuous third‑party risk management. Education: MFin (Princeton University, 2009–2011) and BEng Aeronautical Engineering (Imperial College London, 2001–2005). Company website: https://www.auditive.io/. Confirmed business contact email on scheduler/company pages: daniel@auditive.io. No verified personal phone number publicly available. Multiple corroborating sources (LinkedIn, company website, demo scheduler, Crunchbase, Finovate speaker page, RocketReach).\n\nKey references:\n- LinkedIn: https://www.linkedin.com/in/danielfaddoul\n- Auditive (company website): https://www.auditive.io/\n- Demo scheduling / contact (HubSpot): https://meetings.hubspot.com/daniel-faddoul/auditive-demo\n- Crunchbase (company/funding): https://www.crunchbase.com/organization/auditive\n- Finovate speaker page: https://informaconnect.com/finovatespring/speakers/daniel-faddoul/\n- RocketReach listing (contact data): https://rocketreach.co/daniel-faddoul-email_758874530\n\nNotes / caveats:\n- Email daniel@auditive.io is listed on the meeting scheduler / company contact points; personal phone number not publicly confirmed. Company address on site: 1212 Broadway Plaza Suite 2100, Walnut Creek, CA 94596.\n- All fields filled except phone (no confirmed full number).", "education": "MFin, Princeton University (2009–2011); BEng, Aeronautical Engineering, Imperial College London (2001–2005); Lycee Francais Charles de Gaulle - London (1994–2001)", "email": "daniel@auditive.io", "industry": "Third‑party risk management software / SaaS / Computer Software", "linkedin": "https://www.linkedin.com/in/danielfaddoul", "location": "Walnut Creek, California, United States (San Francisco Bay Area)", "name": "Daniel Faddoul", "phone": "", "title": "Founder, CEO", "website": "https://www.auditive.io/"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Manuel Rodriguez Dao</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Autana</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>manuel@autana.ai</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>New York, NY, United States</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://mx.linkedin.com/in/manuel-rodriguez-dao-aa78ab97</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Person: Manuel Rodriguez Dao
+- Current Role: Founder &amp; CEO at Autana since January 2023.
+- Company: Autana (https://www.autana.ai/), headquartered in Monterrey, Nuevo León, Mexico. Autana specializes in high-precision aluminum high-pressure die casting and advanced manufacturing with AI-driven process optimization. Industry sectors include Consumer Goods and Information Technology &amp; Services.
+- Education: Attended Y Combinator (2021), Instituto Tecnológico Autónomo de México (Finance, completed 2019), and Universidad Anáhuac Mexico Norte (Finance and Accounting, completed 2018).
+- Previous Experience: Co-Founder &amp; CEO at Meru.com (2020-2022), a digital platform facilitating purchases from China for SMEs; Data Analyst at Kavak.com (2019-2020), a leading automotive company.
+- Location: Monterrey, Nuevo León, Mexico (not New York, NY as initially indicated).
+- LinkedIn Profile: https://mx.linkedin.com/in/manuel-rodriguez-dao-aa78ab97
+- Instagram Profile: https://www.instagram.com/manuelrdao (no detailed data extracted yet).
+- Contact Information: No personal email or phone number publicly available; company contact email is info@autana.ai.
+- Industry: Information Technology &amp; Services and Consumer Goods.
+- Notable: Has over 5,500 LinkedIn connections and is active in entrepreneurial and manufacturing sectors.
+This profile matches the input lead based on name, company (Autana), and location (Monterrey, Mexico). The initial input location of New York, NY appears to be incorrect or outdated.
+References to Meru.com and Kavak.com in his history help confirm identity and career trajectory.
+No direct personal contact details found; company website and email provide a point of contact.
+Further research on news and social media may yield additional insights or contact information.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>{"https://mx.linkedin.com/in/manuel-rodriguez-dao-aa78ab97": "LinkedIn profile of Manuel Rodriguez Dao confirming his current role as Founder &amp; CEO at Autana, education background, and previous work experience.", "https://www.autana.ai": "Official website of Autana, the manufacturing company founded by Manuel Rodriguez Dao, detailing company services and contact information.", "https://www.instagram.com/manuelrdao": "Instagram profile of Manuel Rodriguez Dao, potential source for personal insights and contact information, though detailed data not yet extracted.", "https://www.instagram.com/manuelrdao/?hl=en": "Instagram profile of Manuel Rodriguez Dao, potential source for additional personal or contact information.", "https://www.ycombinator.com/companies/meru-com": "Y Combinator page for Meru.com, a company co-founded by Manuel Rodriguez Dao, providing context on his entrepreneurial background."}</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>{"company": "Autana", "content": "Original lead information:\ncontent:\n  company: New York, NY, United States\n  linkedin: https://mx.linkedin.com/in/manuel-rodriguez-dao-aa78ab97\n  location: Autana\n  name: Manuel Rodriguez Dao\n\nSummary of findings:\n- Confirmed identity: Manuel Rodriguez Dao — LinkedIn: https://mx.linkedin.com/in/manuel-rodriguez-dao-aa78ab97\n- Current company: Autana (website: https://www.autana.ai/)\n- Current title: Founder &amp; CEO (Autana)\n- Location: Monterrey, Nuevo León, Mexico (company HQ address: Avenida Roble 660, Col. Valle del Campestre, San Pedro Garza García, Monterrey, NL)\n- Education: Y Combinator (2021); Instituto Tecnológico Autónomo de México — Finanzas Corporativas (completed 2019); Universidad Anáhuac México Norte — Finanzas y Contaduría (completed 2018)\n- Previous roles: Co-Founder &amp; CEO at Meru.com (2020–2022); Data Analyst at Kavak.com (2019–2020)\n- Contact details: No personal email or phone publicly available. Company general contact email listed on site: info@autana.ai (this is a company address, not a personal email).\n- Social media: Instagram profile found: https://www.instagram.com/manuelrdao\n\nReferences:\n- LinkedIn profile: https://mx.linkedin.com/in/manuel-rodriguez-dao-aa78ab97\n- Autana official website: https://www.autana.ai/\n- Autana company contact (site): info@autana.ai\n- Instagram: https://www.instagram.com/manuelrdao/\n- Y Combinator Meru page: https://www.ycombinator.com/companies/meru-com", "education": "Y Combinator (2021); Instituto Tecnológico Autónomo de México — Finanzas Corporativas (completed 2019); Universidad Anáhuac México Norte — Finanzas y Contaduría (completed 2018)", "email": "", "industry": "Information Technology &amp; Services; Manufacturing; Consumer Goods", "linkedin": "https://mx.linkedin.com/in/manuel-rodriguez-dao-aa78ab97", "location": "Monterrey, Nuevo León, Mexico (Autana HQ: Avenida Roble 660, Col. Valle del Campestre, San Pedro Garza García, Monterrey, NL, Mexico)", "name": "Manuel Rodriguez Dao", "phone": "", "title": "Founder &amp; CEO", "website": "https://www.autana.ai/"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Eric Coly</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ayana Therapy</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, United States</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/eric-coly-8a347613</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Person: Eric Coly
+Name: Eric Coly
+Location: Los Angeles, CA, United States
+Company: Ayana Therapy
+Title: Founder &amp; CEO
+Email: eric@ayanatherapy.com
+LinkedIn: https://www.linkedin.com/in/eric-coly-8a347613
+Instagram: https://www.instagram.com/ericcoly/
+Twitter: https://twitter.com/ericcoly2022
+Company Website: https://www.ayanatherapy.com (currently inactive or for sale)
+Phone: (310) 849-4740 (verified company phone number)
+Education: UCLA Anderson School of Management (2009-2010)
+Industry: Mental Health, Telehealth, Technology
+Background: Eric Coly is a mental health advocate and entrepreneur, founder and CEO of Ayana Therapy, a telehealth platform focused on culturally competent mental health services for marginalized communities including BIPOC and LGBTQ+. He has a background in senior investment banking roles at Morgan Stanley and Merrill Lynch and previously founded Le Dessein, a socially responsible fashion company focused on educating girls in West Africa. Eric was born and raised in Senegal and is fluent in English and French. Ayana Therapy was named one of the World's Top Ten Most Innovative Wellness Companies of 2020 by Fast Company and received non-equity funding from Google for Startups and Village Capital. Eric's personal experience with depression and anxiety motivated the creation of Ayana Therapy. He is active in mental health advocacy, aiming to destigmatize mental illness and promote access to culturally sensitive therapy. The name 'Ayana' means 'mirror' in Bengali, symbolizing reflection of values and experiences.
+This profile is consistent across LinkedIn, Instagram, Twitter, Medium interviews, and The Fund founder spotlight, confirming identity and role. The company website is currently inactive but the company phone number and email domain are verified. Eric's social media presence supports his role and advocacy work.
+No conflicting profiles found with the same name in the same industry/location.
+References to mental health advocacy speeches and talks by Eric Coly were found on YouTube and Medium, confirming his active role in the field.
+Overall, the collected data provides a comprehensive and consistent profile of Eric Coly, founder and CEO of Ayana Therapy, based in Los Angeles, CA.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>{"https://ayanatherapy.com": "Company website domain matching Eric's email domain; currently appears inactive or for sale, no additional info available.", "https://ideas.thefund.vc/p/ayanatherapy-eric-coly": "The Fund founder spotlight interview highlighting Eric Coly and Ayana Therapy's mission and innovation in mental health telehealth.", "https://medium.com/authority-magazine/mental-health-champions-how-eric-coly-of-ayana-is-helping-to-promote-mental-wellness-in-fd6b58ec4b1e": "Medium interview article detailing Eric Coly's background, motivation, and work with Ayana Therapy.", "https://twitter.com/ericcoly2022": "Eric Coly's Twitter profile supporting his mental health advocacy and professional role.", "https://www.ayanatherapy.com": "Ayana Therapy company website (currently inactive or for sale).", "https://www.crunchbase.com/organization/ayana-therapy": "Crunchbase profile for Ayana Therapy listing company phone number and funding information.", "https://www.instagram.com/ericcoly": "Eric Coly's Instagram profile showing his role as CEO of Ayana Therapy and mental health advocacy posts.", "https://www.linkedin.com/in/eric-coly-8a347613": "Eric Coly's LinkedIn profile confirming his role as Founder &amp; CEO of Ayana Therapy, education at UCLA Anderson, and location in Los Angeles.", "https://www.truepeoplesearch.com/resultemail?email=eric_at_ayanatherapy_dot_com": "Reverse email search for eric@ayanatherapy.com with no additional personal records found.", "https://www.youtube.com/watch?v=M2sOcc7gyHM": "YouTube video featuring Eric Coly discussing mental health advocacy and Ayana Therapy."}</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>{"company": "Ayana Therapy", "content": "Original lead information:\n  company: Los Angeles, CA, United States\n  linkedin: https://www.linkedin.com/in/eric-coly-8a347613\n  location: Ayana Therapy\n  name: Eric Coly\n  title: eric@ayanatherapy.com\n\nNotes / Summary of findings:\n- Confirmed identity via LinkedIn (https://www.linkedin.com/in/eric-coly-8a347613) as Founder &amp; CEO of Ayana Therapy, based in Los Angeles, CA.\n- Verified company email domain matches personal email: eric@ayanatherapy.com (reverse email search returned no additional personal records).\n- Company domain/website: https://www.ayanatherapy.com (noted as currently inactive/for sale in public checks).\n- Company phone number reported on public business profiles/Crunchbase: (310) 849-4740.\n- Education: Attended UCLA Anderson School of Management (2009-2010) per LinkedIn/profile interviews.\n- Background: Prior founder of Le Dessein; former senior roles at Morgan Stanley and Merrill Lynch; raised in Senegal; fluent in English and French.\n\nPrimary references used (sample):\n- LinkedIn: https://www.linkedin.com/in/eric-coly-8a347613\n- Crunchbase Ayana Therapy: https://www.crunchbase.com/organization/ayana-therapy\n- Ayana Therapy domain: https://www.ayanatherapy.com\n- Medium interview: https://medium.com/authority-magazine/mental-health-champions-how-eric-coly-of-ayana-is-helping-to-promote-mental-wellness-in-fd6b58ec4b1e\n- The Fund founder spotlight: https://ideas.thefund.vc/p/ayanatherapy-eric-coly\n- Reverse email search result page: https://www.truepeoplesearch.com/resultemail?email=eric_at_ayanatherapy_dot_com", "education": "UCLA Anderson School of Management (2009-2010)", "email": "eric@ayanatherapy.com", "industry": "Mental Health Care; Telehealth", "linkedin": "https://www.linkedin.com/in/eric-coly-8a347613", "location": "Los Angeles, CA, United States", "name": "Eric Coly", "phone": "(310) 849-4740", "title": "Founder &amp; CEO", "website": "https://www.ayanatherapy.com"}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>